<commit_message>
5260 - MOQ Table Export
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/MOQTableRMS.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/MOQTableRMS.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BE3DC40-4BA0-4210-B0C6-E2921FEB5AC7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F94508AE-D1B3-439A-9CA2-20F6E5E47F30}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F2BDE59F-50D5-4F91-B73E-5DFBD476F53C}"/>
+    <workbookView xWindow="25545" yWindow="1515" windowWidth="18900" windowHeight="11055" xr2:uid="{F2BDE59F-50D5-4F91-B73E-5DFBD476F53C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="MOQ Tables" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MOQ Tables'!$A$1:$J$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -590,5 +590,13 @@
   <autoFilter ref="A1:J1" xr:uid="{7D4A90C3-D4CB-40BE-BC1C-2D75CA06857E}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader xml:space="preserve">&amp;C  </oddHeader>
+    <oddFooter xml:space="preserve">&amp;C  </oddFooter>
+    <evenHeader xml:space="preserve">&amp;C  </evenHeader>
+    <evenFooter xml:space="preserve">&amp;C  </evenFooter>
+    <firstHeader xml:space="preserve">&amp;C  </firstHeader>
+    <firstFooter xml:space="preserve">&amp;C  </firstFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
IES-806 - PoP Months for RMS in UI, Excel and Word exports
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/MOQTableRMS.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/MOQTableRMS.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F94508AE-D1B3-439A-9CA2-20F6E5E47F30}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29169761-2377-42E0-ADA3-27C27B53C8BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25545" yWindow="1515" windowWidth="18900" windowHeight="11055" xr2:uid="{F2BDE59F-50D5-4F91-B73E-5DFBD476F53C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F2BDE59F-50D5-4F91-B73E-5DFBD476F53C}"/>
   </bookViews>
   <sheets>
     <sheet name="MOQ Tables" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MOQ Tables'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MOQ Tables'!$A$1:$L$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Table Name</t>
   </si>
@@ -69,6 +69,9 @@
   </si>
   <si>
     <t>MOQ Table Custom Field</t>
+  </si>
+  <si>
+    <t>Period of Performance (PoP): Months</t>
   </si>
 </sst>
 </file>
@@ -199,7 +202,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="5" fillId="7" borderId="1" xfId="7" applyNumberFormat="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -211,6 +214,10 @@
     <xf numFmtId="14" fontId="5" fillId="7" borderId="1" xfId="7" applyNumberFormat="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="1" fontId="5" fillId="7" borderId="1" xfId="7" applyNumberFormat="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="genBOE" xfId="7" xr:uid="{3E4869EB-5B79-4DE7-855F-A2B8CADB72D2}"/>
@@ -532,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C581C636-3424-4611-9D2C-375716778AB5}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
@@ -542,13 +549,14 @@
     <col min="5" max="5" width="22.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="42" style="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="41.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="34.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="57.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="60.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="26.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="41.140625" style="8" customWidth="1"/>
+    <col min="9" max="9" width="34.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="57.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="60.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="26.140625" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" s="1" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -570,24 +578,27 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="F2" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1" xr:uid="{7D4A90C3-D4CB-40BE-BC1C-2D75CA06857E}"/>
+  <autoFilter ref="A1:L1" xr:uid="{C581C636-3424-4611-9D2C-375716778AB5}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>

</xml_diff>

<commit_message>
IES-806 - update excel template decimal places
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/MOQTableRMS.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/MOQTableRMS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29169761-2377-42E0-ADA3-27C27B53C8BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{829C4375-3C5C-4588-88B4-6D18FE5CAEA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F2BDE59F-50D5-4F91-B73E-5DFBD476F53C}"/>
+    <workbookView xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15990" xr2:uid="{F2BDE59F-50D5-4F91-B73E-5DFBD476F53C}"/>
   </bookViews>
   <sheets>
     <sheet name="MOQ Tables" sheetId="1" r:id="rId1"/>
@@ -202,7 +202,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="5" fillId="7" borderId="1" xfId="7" applyNumberFormat="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -214,10 +214,9 @@
     <xf numFmtId="14" fontId="5" fillId="7" borderId="1" xfId="7" applyNumberFormat="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="7" borderId="1" xfId="7" applyNumberFormat="1">
+    <xf numFmtId="2" fontId="5" fillId="7" borderId="1" xfId="7" applyNumberFormat="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="genBOE" xfId="7" xr:uid="{3E4869EB-5B79-4DE7-855F-A2B8CADB72D2}"/>
@@ -549,7 +548,7 @@
     <col min="5" max="5" width="22.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="42" style="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="41.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="41.140625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="41.140625" style="4" customWidth="1"/>
     <col min="9" max="9" width="34.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="57.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="60.7109375" style="4" bestFit="1" customWidth="1"/>

</xml_diff>